<commit_message>
refactor: demo_validator 검증 범위 전체 열로 확대, 상수 정의 config.py에 정리
  변경 사항: demo_validator python

app.demo_validator로 실행해야 함
</commit_message>
<xml_diff>
--- a/xlsx_files/2026_기본급여.xlsx
+++ b/xlsx_files/2026_기본급여.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yunjihee/project/한국사회보장정보원_산학협력 프로젝트 과제5_과제 설명자료 및 데이터/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yunjihee/IdeaProjects/ssis-create-excel-table/xlsx_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8318C6E3-FE66-5841-A36D-4C03BFB9C953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B00915-C5DA-5541-AE05-ED9DB13F8F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="8340" windowWidth="18360" windowHeight="16480" activeTab="1" xr2:uid="{A0AAB82A-81F7-4580-BE0A-B18556028628}"/>
+    <workbookView xWindow="1140" yWindow="500" windowWidth="18360" windowHeight="16480" xr2:uid="{A0AAB82A-81F7-4580-BE0A-B18556028628}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11508" uniqueCount="1947">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11418" uniqueCount="1934">
   <si>
     <t>순번</t>
   </si>
@@ -5837,58 +5836,6 @@
   </si>
   <si>
     <t>부적합</t>
-  </si>
-  <si>
-    <t>1등급</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>2등급</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>3등급</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>4등급</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>기본급여(2026) 월한도액</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>기본단가</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>2025 A값</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>초과</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>정부지원금</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">실 본인부담금 </t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>비율 본인부담금</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>본인부담금 상한액(5%)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>본인부담금 상한액(7%)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -5898,7 +5845,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="#,##0_ "/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5928,14 +5875,6 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF3E3E3E"/>
-      <name val="굴림체"/>
-      <family val="2"/>
-      <charset val="129"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -5957,7 +5896,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -5993,173 +5932,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6204,123 +5983,6 @@
     </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6653,7 +6315,7 @@
     <col min="18" max="18" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="28">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -58014,1124 +57676,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B372E972-3C69-954F-823E-A403D654E170}">
-  <dimension ref="A2:S50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
-  <cols>
-    <col min="4" max="4" width="22.5" customWidth="1"/>
-    <col min="13" max="14" width="10.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:19">
-      <c r="A2" s="20" t="s">
-        <v>1938</v>
-      </c>
-      <c r="B2" s="21"/>
-      <c r="D2" s="16" t="s">
-        <v>1939</v>
-      </c>
-      <c r="E2" s="17">
-        <v>17270</v>
-      </c>
-      <c r="G2" s="41">
-        <v>0.5</v>
-      </c>
-      <c r="H2" s="45">
-        <v>0.06</v>
-      </c>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="43"/>
-    </row>
-    <row r="3" spans="1:19">
-      <c r="A3" s="22" t="s">
-        <v>1934</v>
-      </c>
-      <c r="B3" s="23">
-        <v>2041000</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>1940</v>
-      </c>
-      <c r="E3" s="19">
-        <v>3089062</v>
-      </c>
-      <c r="G3" s="46">
-        <v>1</v>
-      </c>
-      <c r="H3" s="47">
-        <v>0.09</v>
-      </c>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-    </row>
-    <row r="4" spans="1:19">
-      <c r="A4" s="22" t="s">
-        <v>1935</v>
-      </c>
-      <c r="B4" s="23">
-        <v>1627000</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1945</v>
-      </c>
-      <c r="E4">
-        <f>ROUNDDOWN(E3*0.05,-2)</f>
-        <v>154400</v>
-      </c>
-      <c r="G4" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="H4" s="47">
-        <v>0.12</v>
-      </c>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
-      <c r="K4" s="44"/>
-    </row>
-    <row r="5" spans="1:19">
-      <c r="A5" s="22" t="s">
-        <v>1936</v>
-      </c>
-      <c r="B5" s="23">
-        <v>1230000</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1946</v>
-      </c>
-      <c r="E5">
-        <f>ROUNDDOWN(E3*0.07,-2)</f>
-        <v>216200</v>
-      </c>
-      <c r="G5" s="24" t="s">
-        <v>1941</v>
-      </c>
-      <c r="H5" s="49">
-        <v>0.15</v>
-      </c>
-      <c r="I5" s="44"/>
-      <c r="J5" s="44"/>
-      <c r="K5" s="44"/>
-    </row>
-    <row r="6" spans="1:19">
-      <c r="A6" s="24" t="s">
-        <v>1937</v>
-      </c>
-      <c r="B6" s="25">
-        <v>815000</v>
-      </c>
-      <c r="N6" s="50"/>
-    </row>
-    <row r="7" spans="1:19">
-      <c r="N7" s="12"/>
-    </row>
-    <row r="8" spans="1:19">
-      <c r="N8" s="12"/>
-    </row>
-    <row r="9" spans="1:19">
-      <c r="A9">
-        <v>1</v>
-      </c>
-      <c r="B9" s="15">
-        <v>8293000</v>
-      </c>
-      <c r="N9" s="12"/>
-    </row>
-    <row r="10" spans="1:19">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10" s="15">
-        <v>7774000</v>
-      </c>
-      <c r="N10" s="12"/>
-    </row>
-    <row r="11" spans="1:19">
-      <c r="A11">
-        <v>3</v>
-      </c>
-      <c r="B11" s="15">
-        <v>7257000</v>
-      </c>
-      <c r="N11" s="12"/>
-    </row>
-    <row r="12" spans="1:19">
-      <c r="A12">
-        <v>4</v>
-      </c>
-      <c r="B12" s="15">
-        <v>6739000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" ht="28">
-      <c r="A13">
-        <v>5</v>
-      </c>
-      <c r="B13" s="15">
-        <v>6221000</v>
-      </c>
-      <c r="D13" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E13" s="36" t="s">
-        <v>4</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>1942</v>
-      </c>
-      <c r="J13" s="31" t="s">
-        <v>1944</v>
-      </c>
-      <c r="K13" s="40" t="s">
-        <v>1943</v>
-      </c>
-      <c r="N13" s="27"/>
-      <c r="O13" s="27"/>
-      <c r="P13" s="27"/>
-      <c r="Q13" s="27"/>
-      <c r="R13" s="27"/>
-      <c r="S13" s="27"/>
-    </row>
-    <row r="14" spans="1:19">
-      <c r="A14">
-        <v>6</v>
-      </c>
-      <c r="B14" s="15">
-        <v>5703000</v>
-      </c>
-      <c r="D14" s="34">
-        <v>1</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H14" s="5">
-        <f>$B$3</f>
-        <v>2041000</v>
-      </c>
-      <c r="I14" s="5">
-        <f>H14-K14</f>
-        <v>2041000</v>
-      </c>
-      <c r="J14" s="32">
-        <v>0</v>
-      </c>
-      <c r="K14" s="15">
-        <f>MIN(J14,$E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="N14" s="28"/>
-      <c r="O14" s="29"/>
-      <c r="P14" s="30"/>
-      <c r="Q14" s="29"/>
-      <c r="R14" s="28"/>
-      <c r="S14" s="28"/>
-    </row>
-    <row r="15" spans="1:19">
-      <c r="A15">
-        <v>7</v>
-      </c>
-      <c r="B15" s="15">
-        <v>5181000</v>
-      </c>
-      <c r="D15" s="35">
-        <v>2</v>
-      </c>
-      <c r="E15" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="5">
-        <f>$B$3</f>
-        <v>2041000</v>
-      </c>
-      <c r="I15" s="5">
-        <f t="shared" ref="I15:I37" si="0">H15-K15</f>
-        <v>2021000</v>
-      </c>
-      <c r="J15" s="33">
-        <v>20000</v>
-      </c>
-      <c r="K15" s="15">
-        <f t="shared" ref="K15:K37" si="1">MIN(J15,$E$4)</f>
-        <v>20000</v>
-      </c>
-      <c r="N15" s="28"/>
-      <c r="O15" s="29"/>
-      <c r="P15" s="30"/>
-      <c r="Q15" s="29"/>
-      <c r="R15" s="28"/>
-      <c r="S15" s="28"/>
-    </row>
-    <row r="16" spans="1:19">
-      <c r="A16">
-        <v>8</v>
-      </c>
-      <c r="B16" s="15">
-        <v>4665000</v>
-      </c>
-      <c r="D16" s="35">
-        <v>3</v>
-      </c>
-      <c r="E16" s="39" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="5">
-        <f t="shared" ref="H15:H19" si="2">$B$3</f>
-        <v>2041000</v>
-      </c>
-      <c r="I16" s="5">
-        <f t="shared" si="0"/>
-        <v>1918600</v>
-      </c>
-      <c r="J16" s="33">
-        <f>ROUNDDOWN($B$3*H2,-2)</f>
-        <v>122400</v>
-      </c>
-      <c r="K16" s="15">
-        <f t="shared" si="1"/>
-        <v>122400</v>
-      </c>
-      <c r="N16" s="28"/>
-      <c r="O16" s="29"/>
-      <c r="P16" s="30"/>
-      <c r="Q16" s="29"/>
-      <c r="R16" s="28"/>
-      <c r="S16" s="28"/>
-    </row>
-    <row r="17" spans="1:19">
-      <c r="A17">
-        <v>9</v>
-      </c>
-      <c r="B17" s="15">
-        <v>4148000</v>
-      </c>
-      <c r="D17" s="35">
-        <v>4</v>
-      </c>
-      <c r="E17" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H17" s="5">
-        <f t="shared" si="2"/>
-        <v>2041000</v>
-      </c>
-      <c r="I17" s="5">
-        <f t="shared" si="0"/>
-        <v>1886600</v>
-      </c>
-      <c r="J17" s="33">
-        <f t="shared" ref="J17:J19" si="3">ROUNDDOWN($B$3*H3,-2)</f>
-        <v>183600</v>
-      </c>
-      <c r="K17" s="15">
-        <f t="shared" si="1"/>
-        <v>154400</v>
-      </c>
-      <c r="N17" s="28"/>
-      <c r="O17" s="29"/>
-      <c r="P17" s="30"/>
-      <c r="Q17" s="29"/>
-      <c r="R17" s="28"/>
-      <c r="S17" s="28"/>
-    </row>
-    <row r="18" spans="1:19">
-      <c r="A18">
-        <v>10</v>
-      </c>
-      <c r="B18" s="15">
-        <v>3629000</v>
-      </c>
-      <c r="D18" s="35">
-        <v>5</v>
-      </c>
-      <c r="E18" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H18" s="5">
-        <f t="shared" si="2"/>
-        <v>2041000</v>
-      </c>
-      <c r="I18" s="5">
-        <f t="shared" si="0"/>
-        <v>1886600</v>
-      </c>
-      <c r="J18" s="33">
-        <f t="shared" si="3"/>
-        <v>244900</v>
-      </c>
-      <c r="K18" s="15">
-        <f>MIN(J18,$E$4)</f>
-        <v>154400</v>
-      </c>
-      <c r="N18" s="28"/>
-      <c r="O18" s="29"/>
-      <c r="P18" s="30"/>
-      <c r="Q18" s="29"/>
-      <c r="R18" s="28"/>
-      <c r="S18" s="28"/>
-    </row>
-    <row r="19" spans="1:19">
-      <c r="A19">
-        <v>11</v>
-      </c>
-      <c r="B19" s="15">
-        <v>3112000</v>
-      </c>
-      <c r="D19" s="35">
-        <v>6</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" s="5">
-        <f t="shared" si="2"/>
-        <v>2041000</v>
-      </c>
-      <c r="I19" s="5">
-        <f t="shared" si="0"/>
-        <v>1886600</v>
-      </c>
-      <c r="J19" s="33">
-        <f>ROUNDDOWN($B$3*H5,-2)</f>
-        <v>306100</v>
-      </c>
-      <c r="K19" s="15">
-        <f t="shared" si="1"/>
-        <v>154400</v>
-      </c>
-      <c r="N19" s="28"/>
-      <c r="O19" s="29"/>
-      <c r="P19" s="30"/>
-      <c r="Q19" s="29"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
-    </row>
-    <row r="20" spans="1:19" ht="18" thickBot="1">
-      <c r="A20">
-        <v>12</v>
-      </c>
-      <c r="B20" s="15">
-        <v>2593000</v>
-      </c>
-      <c r="D20" s="35">
-        <v>7</v>
-      </c>
-      <c r="E20" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H20" s="12">
-        <f>$B$4</f>
-        <v>1627000</v>
-      </c>
-      <c r="I20" s="5">
-        <f t="shared" si="0"/>
-        <v>1627000</v>
-      </c>
-      <c r="J20" s="32">
-        <v>0</v>
-      </c>
-      <c r="K20" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M20" s="51"/>
-      <c r="N20" s="52"/>
-      <c r="O20" s="53"/>
-      <c r="P20" s="30"/>
-      <c r="Q20" s="29"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
-    </row>
-    <row r="21" spans="1:19">
-      <c r="A21">
-        <v>13</v>
-      </c>
-      <c r="B21" s="15">
-        <v>2076000</v>
-      </c>
-      <c r="D21" s="35">
-        <v>8</v>
-      </c>
-      <c r="E21" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H21" s="12">
-        <f t="shared" ref="H21:H25" si="4">$B$4</f>
-        <v>1627000</v>
-      </c>
-      <c r="I21" s="5">
-        <f t="shared" si="0"/>
-        <v>1607000</v>
-      </c>
-      <c r="J21" s="33">
-        <v>20000</v>
-      </c>
-      <c r="K21" s="15">
-        <f t="shared" si="1"/>
-        <v>20000</v>
-      </c>
-      <c r="N21" s="28"/>
-      <c r="O21" s="29"/>
-      <c r="P21" s="30"/>
-      <c r="Q21" s="29"/>
-      <c r="R21" s="28"/>
-      <c r="S21" s="28"/>
-    </row>
-    <row r="22" spans="1:19">
-      <c r="A22">
-        <v>14</v>
-      </c>
-      <c r="B22" s="15">
-        <v>1558000</v>
-      </c>
-      <c r="D22" s="35">
-        <v>9</v>
-      </c>
-      <c r="E22" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H22" s="12">
-        <f t="shared" si="4"/>
-        <v>1627000</v>
-      </c>
-      <c r="I22" s="5">
-        <f t="shared" si="0"/>
-        <v>1529400</v>
-      </c>
-      <c r="J22" s="33">
-        <f>ROUNDDOWN($B$4*H2,-2)</f>
-        <v>97600</v>
-      </c>
-      <c r="K22" s="15">
-        <f t="shared" si="1"/>
-        <v>97600</v>
-      </c>
-      <c r="N22" s="28"/>
-      <c r="O22" s="29"/>
-      <c r="P22" s="30"/>
-      <c r="Q22" s="29"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-    </row>
-    <row r="23" spans="1:19">
-      <c r="A23">
-        <v>15</v>
-      </c>
-      <c r="B23" s="15">
-        <v>1040000</v>
-      </c>
-      <c r="D23" s="35">
-        <v>10</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="G23" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H23" s="12">
-        <f t="shared" si="4"/>
-        <v>1627000</v>
-      </c>
-      <c r="I23" s="5">
-        <f t="shared" si="0"/>
-        <v>1480600</v>
-      </c>
-      <c r="J23" s="33">
-        <f t="shared" ref="J23:J26" si="5">ROUNDDOWN($B$4*H3,-2)</f>
-        <v>146400</v>
-      </c>
-      <c r="K23" s="15">
-        <f t="shared" si="1"/>
-        <v>146400</v>
-      </c>
-      <c r="N23" s="28"/>
-      <c r="O23" s="29"/>
-      <c r="P23" s="30"/>
-      <c r="Q23" s="29"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="28"/>
-    </row>
-    <row r="24" spans="1:19">
-      <c r="D24" s="35">
-        <v>11</v>
-      </c>
-      <c r="E24" s="39" t="s">
-        <v>49</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="G24" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H24" s="12">
-        <f t="shared" si="4"/>
-        <v>1627000</v>
-      </c>
-      <c r="I24" s="5">
-        <f t="shared" si="0"/>
-        <v>1472600</v>
-      </c>
-      <c r="J24" s="33">
-        <f t="shared" si="5"/>
-        <v>195200</v>
-      </c>
-      <c r="K24" s="15">
-        <f t="shared" si="1"/>
-        <v>154400</v>
-      </c>
-      <c r="N24" s="28"/>
-      <c r="O24" s="29"/>
-      <c r="P24" s="30"/>
-      <c r="Q24" s="29"/>
-      <c r="R24" s="28"/>
-      <c r="S24" s="28"/>
-    </row>
-    <row r="25" spans="1:19">
-      <c r="D25" s="35">
-        <v>12</v>
-      </c>
-      <c r="E25" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="G25" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H25" s="12">
-        <f t="shared" si="4"/>
-        <v>1627000</v>
-      </c>
-      <c r="I25" s="5">
-        <f t="shared" si="0"/>
-        <v>1472600</v>
-      </c>
-      <c r="J25" s="33">
-        <f t="shared" si="5"/>
-        <v>244000</v>
-      </c>
-      <c r="K25" s="15">
-        <f t="shared" si="1"/>
-        <v>154400</v>
-      </c>
-      <c r="N25" s="28"/>
-      <c r="O25" s="29"/>
-      <c r="P25" s="30"/>
-      <c r="Q25" s="29"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-    </row>
-    <row r="26" spans="1:19">
-      <c r="D26" s="35">
-        <v>13</v>
-      </c>
-      <c r="E26" s="39" t="s">
-        <v>53</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G26" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H26" s="12">
-        <f>$B$5</f>
-        <v>1230000</v>
-      </c>
-      <c r="I26" s="5">
-        <f t="shared" si="0"/>
-        <v>1230000</v>
-      </c>
-      <c r="J26" s="33">
-        <v>0</v>
-      </c>
-      <c r="K26" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N26" s="28"/>
-      <c r="O26" s="29"/>
-      <c r="P26" s="30"/>
-      <c r="Q26" s="29"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28"/>
-    </row>
-    <row r="27" spans="1:19">
-      <c r="D27" s="35">
-        <v>14</v>
-      </c>
-      <c r="E27" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G27" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H27" s="12">
-        <f t="shared" ref="H27:H31" si="6">$B$5</f>
-        <v>1230000</v>
-      </c>
-      <c r="I27" s="5">
-        <f t="shared" si="0"/>
-        <v>1210000</v>
-      </c>
-      <c r="J27" s="33">
-        <f>J15</f>
-        <v>20000</v>
-      </c>
-      <c r="K27" s="15">
-        <f t="shared" si="1"/>
-        <v>20000</v>
-      </c>
-      <c r="N27" s="28"/>
-      <c r="O27" s="29"/>
-      <c r="P27" s="30"/>
-      <c r="Q27" s="29"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28"/>
-    </row>
-    <row r="28" spans="1:19">
-      <c r="D28" s="35">
-        <v>15</v>
-      </c>
-      <c r="E28" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H28" s="12">
-        <f t="shared" si="6"/>
-        <v>1230000</v>
-      </c>
-      <c r="I28" s="5">
-        <f t="shared" si="0"/>
-        <v>1156200</v>
-      </c>
-      <c r="J28" s="33">
-        <f>ROUNDDOWN($B$5*H2,-2)</f>
-        <v>73800</v>
-      </c>
-      <c r="K28" s="15">
-        <f t="shared" si="1"/>
-        <v>73800</v>
-      </c>
-      <c r="N28" s="28"/>
-      <c r="O28" s="29"/>
-      <c r="P28" s="30"/>
-      <c r="Q28" s="29"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="28"/>
-    </row>
-    <row r="29" spans="1:19">
-      <c r="D29" s="35">
-        <v>16</v>
-      </c>
-      <c r="E29" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H29" s="12">
-        <f t="shared" si="6"/>
-        <v>1230000</v>
-      </c>
-      <c r="I29" s="5">
-        <f t="shared" si="0"/>
-        <v>1119300</v>
-      </c>
-      <c r="J29" s="33">
-        <f t="shared" ref="J29:J31" si="7">ROUNDDOWN($B$5*H3,-2)</f>
-        <v>110700</v>
-      </c>
-      <c r="K29" s="15">
-        <f t="shared" si="1"/>
-        <v>110700</v>
-      </c>
-      <c r="N29" s="28"/>
-      <c r="O29" s="29"/>
-      <c r="P29" s="30"/>
-      <c r="Q29" s="29"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
-    </row>
-    <row r="30" spans="1:19">
-      <c r="D30" s="35">
-        <v>17</v>
-      </c>
-      <c r="E30" s="39" t="s">
-        <v>61</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H30" s="12">
-        <f t="shared" si="6"/>
-        <v>1230000</v>
-      </c>
-      <c r="I30" s="5">
-        <f t="shared" si="0"/>
-        <v>1082400</v>
-      </c>
-      <c r="J30" s="33">
-        <f t="shared" si="7"/>
-        <v>147600</v>
-      </c>
-      <c r="K30" s="15">
-        <f t="shared" si="1"/>
-        <v>147600</v>
-      </c>
-      <c r="N30" s="28"/>
-      <c r="O30" s="29"/>
-      <c r="P30" s="30"/>
-      <c r="Q30" s="29"/>
-      <c r="R30" s="28"/>
-      <c r="S30" s="28"/>
-    </row>
-    <row r="31" spans="1:19">
-      <c r="D31" s="35">
-        <v>18</v>
-      </c>
-      <c r="E31" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="G31" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H31" s="12">
-        <f t="shared" si="6"/>
-        <v>1230000</v>
-      </c>
-      <c r="I31" s="5">
-        <f t="shared" si="0"/>
-        <v>1075600</v>
-      </c>
-      <c r="J31" s="33">
-        <f t="shared" si="7"/>
-        <v>184500</v>
-      </c>
-      <c r="K31" s="15">
-        <f t="shared" si="1"/>
-        <v>154400</v>
-      </c>
-      <c r="N31" s="28"/>
-      <c r="O31" s="29"/>
-      <c r="P31" s="30"/>
-      <c r="Q31" s="29"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-    </row>
-    <row r="32" spans="1:19">
-      <c r="D32" s="35">
-        <v>19</v>
-      </c>
-      <c r="E32" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G32" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H32" s="12">
-        <f>$B$6</f>
-        <v>815000</v>
-      </c>
-      <c r="I32" s="5">
-        <f t="shared" si="0"/>
-        <v>815000</v>
-      </c>
-      <c r="J32" s="33">
-        <v>0</v>
-      </c>
-      <c r="K32" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N32" s="28"/>
-      <c r="O32" s="29"/>
-      <c r="P32" s="30"/>
-      <c r="Q32" s="29"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-    </row>
-    <row r="33" spans="4:19">
-      <c r="D33" s="35">
-        <v>20</v>
-      </c>
-      <c r="E33" s="38" t="s">
-        <v>67</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="G33" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H33" s="12">
-        <f t="shared" ref="H33:H37" si="8">$B$6</f>
-        <v>815000</v>
-      </c>
-      <c r="I33" s="5">
-        <f t="shared" si="0"/>
-        <v>795000</v>
-      </c>
-      <c r="J33" s="33">
-        <f>J15</f>
-        <v>20000</v>
-      </c>
-      <c r="K33" s="15">
-        <f t="shared" si="1"/>
-        <v>20000</v>
-      </c>
-      <c r="N33" s="28"/>
-      <c r="O33" s="29"/>
-      <c r="P33" s="30"/>
-      <c r="Q33" s="29"/>
-      <c r="R33" s="28"/>
-      <c r="S33" s="28"/>
-    </row>
-    <row r="34" spans="4:19">
-      <c r="D34" s="35">
-        <v>21</v>
-      </c>
-      <c r="E34" s="39" t="s">
-        <v>69</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="G34" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H34" s="12">
-        <f t="shared" si="8"/>
-        <v>815000</v>
-      </c>
-      <c r="I34" s="5">
-        <f t="shared" si="0"/>
-        <v>766100</v>
-      </c>
-      <c r="J34" s="33">
-        <f>ROUNDDOWN($B$6*H2,-2)</f>
-        <v>48900</v>
-      </c>
-      <c r="K34" s="15">
-        <f t="shared" si="1"/>
-        <v>48900</v>
-      </c>
-      <c r="N34" s="28"/>
-      <c r="O34" s="29"/>
-      <c r="P34" s="30"/>
-      <c r="Q34" s="29"/>
-      <c r="R34" s="28"/>
-      <c r="S34" s="28"/>
-    </row>
-    <row r="35" spans="4:19" ht="18" thickBot="1">
-      <c r="D35" s="35">
-        <v>22</v>
-      </c>
-      <c r="E35" s="38" t="s">
-        <v>71</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H35" s="12">
-        <f t="shared" si="8"/>
-        <v>815000</v>
-      </c>
-      <c r="I35" s="5">
-        <f t="shared" si="0"/>
-        <v>741700</v>
-      </c>
-      <c r="J35" s="33">
-        <f t="shared" ref="J35:J37" si="9">ROUNDDOWN($B$6*H3,-2)</f>
-        <v>73300</v>
-      </c>
-      <c r="K35" s="15">
-        <f t="shared" si="1"/>
-        <v>73300</v>
-      </c>
-      <c r="M35" s="51"/>
-      <c r="N35" s="52"/>
-      <c r="O35" s="53"/>
-      <c r="P35" s="30"/>
-      <c r="Q35" s="29"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
-    </row>
-    <row r="36" spans="4:19">
-      <c r="D36" s="35">
-        <v>23</v>
-      </c>
-      <c r="E36" s="39" t="s">
-        <v>73</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="G36" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H36" s="12">
-        <f t="shared" si="8"/>
-        <v>815000</v>
-      </c>
-      <c r="I36" s="5">
-        <f t="shared" si="0"/>
-        <v>717200</v>
-      </c>
-      <c r="J36" s="33">
-        <f t="shared" si="9"/>
-        <v>97800</v>
-      </c>
-      <c r="K36" s="15">
-        <f t="shared" si="1"/>
-        <v>97800</v>
-      </c>
-      <c r="N36" s="28"/>
-      <c r="O36" s="29"/>
-      <c r="P36" s="30"/>
-      <c r="Q36" s="29"/>
-      <c r="R36" s="28"/>
-      <c r="S36" s="28"/>
-    </row>
-    <row r="37" spans="4:19">
-      <c r="D37" s="35">
-        <v>24</v>
-      </c>
-      <c r="E37" s="38" t="s">
-        <v>75</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="G37" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H37" s="12">
-        <f t="shared" si="8"/>
-        <v>815000</v>
-      </c>
-      <c r="I37" s="5">
-        <f t="shared" si="0"/>
-        <v>692800</v>
-      </c>
-      <c r="J37" s="33">
-        <f t="shared" si="9"/>
-        <v>122200</v>
-      </c>
-      <c r="K37" s="15">
-        <f t="shared" si="1"/>
-        <v>122200</v>
-      </c>
-      <c r="N37" s="28"/>
-      <c r="O37" s="29"/>
-      <c r="P37" s="30"/>
-      <c r="Q37" s="29"/>
-      <c r="R37" s="28"/>
-      <c r="S37" s="28"/>
-    </row>
-    <row r="50" spans="13:15" ht="18" thickBot="1">
-      <c r="M50" s="51"/>
-      <c r="N50" s="51"/>
-      <c r="O50" s="51"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>